<commit_message>
fixing the nis issues
</commit_message>
<xml_diff>
--- a/public/templates/template_import_santri.xlsx
+++ b/public/templates/template_import_santri.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tamam\Herd\sia\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{601119E6-5F72-4931-A5A4-E9A62608E1CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0B92B58-1DA5-4FFD-951D-2F5D1EB995FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{E4F09937-6EAF-4319-B60C-264F9E558CD0}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>NIS</t>
   </si>
@@ -43,9 +43,6 @@
     <t>No Telp Wali</t>
   </si>
   <si>
-    <t>Email</t>
-  </si>
-  <si>
     <t>Muhammad Fulan</t>
   </si>
   <si>
@@ -53,9 +50,6 @@
   </si>
   <si>
     <t>Fulan Ahmad</t>
-  </si>
-  <si>
-    <t>fulan@gmail.com</t>
   </si>
   <si>
     <t>&gt;&gt; Ini Baris Contoh, Hapus baris ini jika hendak import</t>
@@ -925,7 +919,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75A8225A-E4DD-40BB-94FF-6DBA67E8AD84}">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6" bestFit="1" customWidth="1"/>
@@ -936,7 +930,7 @@
     <col min="7" max="7" width="13.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -958,37 +952,31 @@
       <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>20002</v>
+      </c>
+      <c r="B2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>21008</v>
-      </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>8</v>
-      </c>
-      <c r="C2" t="s">
-        <v>9</v>
       </c>
       <c r="D2" s="1">
         <v>53191</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H2" t="s">
         <v>10</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H2" t="s">
-        <v>11</v>
-      </c>
-      <c r="I2" t="s">
-        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>